<commit_message>
Deploying to gh-pages from  @ 0a7adcad0f596ee66b811e598d43dc6cd2976596 🚀
</commit_message>
<xml_diff>
--- a/api/clv2/xlsx/en/SectorGroup.xlsx
+++ b/api/clv2/xlsx/en/SectorGroup.xlsx
@@ -28,15 +28,15 @@
     <t>codeforiati:sector-name</t>
   </si>
   <si>
+    <t>codeforiati:category-name</t>
+  </si>
+  <si>
     <t>codeforiati:category-code</t>
   </si>
   <si>
     <t>codeforiati:sector-code</t>
   </si>
   <si>
-    <t>codeforiati:category-name</t>
-  </si>
-  <si>
     <t>110</t>
   </si>
   <si>
@@ -49,15 +49,15 @@
     <t>Advanced technical and managerial training</t>
   </si>
   <si>
+    <t>Post-Secondary Education</t>
+  </si>
+  <si>
     <t>114</t>
   </si>
   <si>
     <t>11430</t>
   </si>
   <si>
-    <t>Post-Secondary Education</t>
-  </si>
-  <si>
     <t>120</t>
   </si>
   <si>
@@ -67,15 +67,15 @@
     <t>Research for prevention and control of NCDs</t>
   </si>
   <si>
+    <t>Non-communicable diseases (NCDs)</t>
+  </si>
+  <si>
     <t>123</t>
   </si>
   <si>
     <t>12382</t>
   </si>
   <si>
-    <t>Non-communicable diseases (NCDs)</t>
-  </si>
-  <si>
     <t>130</t>
   </si>
   <si>
@@ -109,15 +109,15 @@
     <t>Child soldiers (prevention and demobilisation)</t>
   </si>
   <si>
+    <t>Conflict, Peace &amp; Security</t>
+  </si>
+  <si>
     <t>152</t>
   </si>
   <si>
     <t>15261</t>
   </si>
   <si>
-    <t>Conflict, Peace &amp; Security</t>
-  </si>
-  <si>
     <t>160</t>
   </si>
   <si>
@@ -163,15 +163,15 @@
     <t>Electric mobility infrastructures</t>
   </si>
   <si>
+    <t>Energy distribution</t>
+  </si>
+  <si>
     <t>236</t>
   </si>
   <si>
     <t>23642</t>
   </si>
   <si>
-    <t>Energy distribution</t>
-  </si>
-  <si>
     <t>240</t>
   </si>
   <si>
@@ -205,15 +205,15 @@
     <t>Fishery services</t>
   </si>
   <si>
+    <t>Fishing</t>
+  </si>
+  <si>
     <t>313</t>
   </si>
   <si>
     <t>31391</t>
   </si>
   <si>
-    <t>Fishing</t>
-  </si>
-  <si>
     <t>320</t>
   </si>
   <si>
@@ -223,13 +223,13 @@
     <t>Construction policy and administrative management</t>
   </si>
   <si>
+    <t>Construction</t>
+  </si>
+  <si>
     <t>323</t>
   </si>
   <si>
     <t>32310</t>
-  </si>
-  <si>
-    <t>Construction</t>
   </si>
   <si>
     <t>331</t>
@@ -815,13 +815,13 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -838,13 +838,13 @@
         <v>26</v>
       </c>
       <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
         <v>24</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>27</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -884,13 +884,13 @@
         <v>36</v>
       </c>
       <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
         <v>34</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>37</v>
-      </c>
-      <c r="G7" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -907,13 +907,13 @@
         <v>40</v>
       </c>
       <c r="E8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" t="s">
         <v>38</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>41</v>
-      </c>
-      <c r="G8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -930,13 +930,13 @@
         <v>44</v>
       </c>
       <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" t="s">
         <v>42</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>45</v>
-      </c>
-      <c r="G9" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -976,13 +976,13 @@
         <v>54</v>
       </c>
       <c r="E11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" t="s">
         <v>52</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>55</v>
-      </c>
-      <c r="G11" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -999,13 +999,13 @@
         <v>58</v>
       </c>
       <c r="E12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" t="s">
         <v>56</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>59</v>
-      </c>
-      <c r="G12" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1068,13 +1068,13 @@
         <v>74</v>
       </c>
       <c r="E15" t="s">
+        <v>73</v>
+      </c>
+      <c r="F15" t="s">
         <v>72</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>75</v>
-      </c>
-      <c r="G15" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1091,13 +1091,13 @@
         <v>78</v>
       </c>
       <c r="E16" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" t="s">
         <v>76</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>79</v>
-      </c>
-      <c r="G16" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1114,13 +1114,13 @@
         <v>82</v>
       </c>
       <c r="E17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
         <v>80</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>83</v>
-      </c>
-      <c r="G17" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1137,13 +1137,13 @@
         <v>86</v>
       </c>
       <c r="E18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>87</v>
-      </c>
-      <c r="G18" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1160,13 +1160,13 @@
         <v>90</v>
       </c>
       <c r="E19" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" t="s">
         <v>88</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>91</v>
-      </c>
-      <c r="G19" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1183,13 +1183,13 @@
         <v>94</v>
       </c>
       <c r="E20" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" t="s">
         <v>92</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>95</v>
-      </c>
-      <c r="G20" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1206,13 +1206,13 @@
         <v>98</v>
       </c>
       <c r="E21" t="s">
+        <v>97</v>
+      </c>
+      <c r="F21" t="s">
         <v>96</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>99</v>
-      </c>
-      <c r="G21" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1229,13 +1229,13 @@
         <v>102</v>
       </c>
       <c r="E22" t="s">
+        <v>101</v>
+      </c>
+      <c r="F22" t="s">
         <v>100</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>103</v>
-      </c>
-      <c r="G22" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1252,13 +1252,13 @@
         <v>106</v>
       </c>
       <c r="E23" t="s">
+        <v>105</v>
+      </c>
+      <c r="F23" t="s">
         <v>104</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>107</v>
-      </c>
-      <c r="G23" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1275,13 +1275,13 @@
         <v>110</v>
       </c>
       <c r="E24" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" t="s">
         <v>108</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>111</v>
-      </c>
-      <c r="G24" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1298,13 +1298,13 @@
         <v>114</v>
       </c>
       <c r="E25" t="s">
+        <v>113</v>
+      </c>
+      <c r="F25" t="s">
         <v>112</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>115</v>
-      </c>
-      <c r="G25" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1321,13 +1321,13 @@
         <v>118</v>
       </c>
       <c r="E26" t="s">
+        <v>117</v>
+      </c>
+      <c r="F26" t="s">
         <v>116</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>119</v>
-      </c>
-      <c r="G26" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1344,13 +1344,13 @@
         <v>122</v>
       </c>
       <c r="E27" t="s">
+        <v>121</v>
+      </c>
+      <c r="F27" t="s">
         <v>120</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>123</v>
-      </c>
-      <c r="G27" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1367,13 +1367,13 @@
         <v>126</v>
       </c>
       <c r="E28" t="s">
+        <v>125</v>
+      </c>
+      <c r="F28" t="s">
         <v>124</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>127</v>
-      </c>
-      <c r="G28" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ ef85588f12a75e1b964523c909e0ff79b4a3e743 🚀
</commit_message>
<xml_diff>
--- a/api/clv2/xlsx/en/SectorGroup.xlsx
+++ b/api/clv2/xlsx/en/SectorGroup.xlsx
@@ -25,18 +25,18 @@
     <t>status</t>
   </si>
   <si>
+    <t>codeforiati:group-code</t>
+  </si>
+  <si>
+    <t>codeforiati:category-name</t>
+  </si>
+  <si>
     <t>codeforiati:category-code</t>
   </si>
   <si>
     <t>codeforiati:group-name</t>
   </si>
   <si>
-    <t>codeforiati:category-name</t>
-  </si>
-  <si>
-    <t>codeforiati:group-code</t>
-  </si>
-  <si>
     <t>11110</t>
   </si>
   <si>
@@ -46,18 +46,18 @@
     <t>active</t>
   </si>
   <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>Education, Level Unspecified</t>
+  </si>
+  <si>
     <t>111</t>
   </si>
   <si>
     <t>Education</t>
   </si>
   <si>
-    <t>Education, Level Unspecified</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
     <t>11120</t>
   </si>
   <si>
@@ -82,12 +82,12 @@
     <t>Primary education</t>
   </si>
   <si>
+    <t>Basic Education</t>
+  </si>
+  <si>
     <t>112</t>
   </si>
   <si>
-    <t>Basic Education</t>
-  </si>
-  <si>
     <t>11230</t>
   </si>
   <si>
@@ -112,12 +112,12 @@
     <t>Secondary education</t>
   </si>
   <si>
+    <t>Secondary Education</t>
+  </si>
+  <si>
     <t>113</t>
   </si>
   <si>
-    <t>Secondary Education</t>
-  </si>
-  <si>
     <t>11330</t>
   </si>
   <si>
@@ -130,12 +130,12 @@
     <t>Higher education</t>
   </si>
   <si>
+    <t>Post-Secondary Education</t>
+  </si>
+  <si>
     <t>114</t>
   </si>
   <si>
-    <t>Post-Secondary Education</t>
-  </si>
-  <si>
     <t>11430</t>
   </si>
   <si>
@@ -148,18 +148,18 @@
     <t>Health policy and administrative management</t>
   </si>
   <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>Health, General</t>
+  </si>
+  <si>
     <t>121</t>
   </si>
   <si>
     <t>Health</t>
   </si>
   <si>
-    <t>Health, General</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
     <t>12181</t>
   </si>
   <si>
@@ -184,12 +184,12 @@
     <t>Basic health care</t>
   </si>
   <si>
+    <t>Basic Health</t>
+  </si>
+  <si>
     <t>122</t>
   </si>
   <si>
-    <t>Basic Health</t>
-  </si>
-  <si>
     <t>12230</t>
   </si>
   <si>
@@ -238,12 +238,12 @@
     <t>NCDs control, general</t>
   </si>
   <si>
+    <t>Non-communicable diseases (NCDs)</t>
+  </si>
+  <si>
     <t>123</t>
   </si>
   <si>
-    <t>Non-communicable diseases (NCDs)</t>
-  </si>
-  <si>
     <t>12320</t>
   </si>
   <si>
@@ -388,18 +388,18 @@
     <t>Public sector policy and administrative management</t>
   </si>
   <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>Government &amp; Civil Society-general</t>
+  </si>
+  <si>
     <t>151</t>
   </si>
   <si>
     <t>Government &amp; Civil Society</t>
   </si>
   <si>
-    <t>Government &amp; Civil Society-general</t>
-  </si>
-  <si>
-    <t>150</t>
-  </si>
-  <si>
     <t>15111</t>
   </si>
   <si>
@@ -496,12 +496,12 @@
     <t>Security system management and reform</t>
   </si>
   <si>
+    <t>Conflict, Peace &amp; Security</t>
+  </si>
+  <si>
     <t>152</t>
   </si>
   <si>
-    <t>Conflict, Peace &amp; Security</t>
-  </si>
-  <si>
     <t>15220</t>
   </si>
   <si>
@@ -688,18 +688,18 @@
     <t>Energy policy and administrative management</t>
   </si>
   <si>
+    <t>230</t>
+  </si>
+  <si>
+    <t>Energy Policy</t>
+  </si>
+  <si>
     <t>231</t>
   </si>
   <si>
     <t>Energy</t>
   </si>
   <si>
-    <t>Energy Policy</t>
-  </si>
-  <si>
-    <t>230</t>
-  </si>
-  <si>
     <t>23181</t>
   </si>
   <si>
@@ -724,12 +724,12 @@
     <t>Energy generation, renewable sources - multiple technologies</t>
   </si>
   <si>
+    <t>Energy generation, renewable sources</t>
+  </si>
+  <si>
     <t>232</t>
   </si>
   <si>
-    <t>Energy generation, renewable sources</t>
-  </si>
-  <si>
     <t>23220</t>
   </si>
   <si>
@@ -784,12 +784,12 @@
     <t>Energy generation, non-renewable sources, unspecified</t>
   </si>
   <si>
+    <t>Energy generation, non-renewable sources</t>
+  </si>
+  <si>
     <t>233</t>
   </si>
   <si>
-    <t>Energy generation, non-renewable sources</t>
-  </si>
-  <si>
     <t>23320</t>
   </si>
   <si>
@@ -826,36 +826,36 @@
     <t>Hybrid energy electric power plants</t>
   </si>
   <si>
+    <t>Hybrid energy plants</t>
+  </si>
+  <si>
     <t>234</t>
   </si>
   <si>
-    <t>Hybrid energy plants</t>
-  </si>
-  <si>
     <t>23510</t>
   </si>
   <si>
     <t>Nuclear energy electric power plants and nuclear safety</t>
   </si>
   <si>
+    <t>Nuclear energy plants</t>
+  </si>
+  <si>
     <t>235</t>
   </si>
   <si>
-    <t>Nuclear energy plants</t>
-  </si>
-  <si>
     <t>23610</t>
   </si>
   <si>
     <t>Heat plants</t>
   </si>
   <si>
+    <t>Energy distribution</t>
+  </si>
+  <si>
     <t>236</t>
   </si>
   <si>
-    <t>Energy distribution</t>
-  </si>
-  <si>
     <t>23620</t>
   </si>
   <si>
@@ -970,18 +970,18 @@
     <t>Agricultural policy and administrative management</t>
   </si>
   <si>
+    <t>310</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
     <t>311</t>
   </si>
   <si>
     <t>Agriculture, Forestry, Fishing</t>
   </si>
   <si>
-    <t>Agriculture</t>
-  </si>
-  <si>
-    <t>310</t>
-  </si>
-  <si>
     <t>31120</t>
   </si>
   <si>
@@ -1090,12 +1090,12 @@
     <t>Forestry policy and administrative management</t>
   </si>
   <si>
+    <t>Forestry</t>
+  </si>
+  <si>
     <t>312</t>
   </si>
   <si>
-    <t>Forestry</t>
-  </si>
-  <si>
     <t>31220</t>
   </si>
   <si>
@@ -1132,12 +1132,12 @@
     <t>Fishing policy and administrative management</t>
   </si>
   <si>
+    <t>Fishing</t>
+  </si>
+  <si>
     <t>313</t>
   </si>
   <si>
-    <t>Fishing</t>
-  </si>
-  <si>
     <t>31320</t>
   </si>
   <si>
@@ -1168,18 +1168,18 @@
     <t>Industrial policy and administrative management</t>
   </si>
   <si>
+    <t>320</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
     <t>321</t>
   </si>
   <si>
     <t>Industry, Mining, Construction</t>
   </si>
   <si>
-    <t>Industry</t>
-  </si>
-  <si>
-    <t>320</t>
-  </si>
-  <si>
     <t>32120</t>
   </si>
   <si>
@@ -1294,12 +1294,12 @@
     <t>Mineral/mining policy and administrative management</t>
   </si>
   <si>
+    <t>Mineral Resources &amp; Mining</t>
+  </si>
+  <si>
     <t>322</t>
   </si>
   <si>
-    <t>Mineral Resources &amp; Mining</t>
-  </si>
-  <si>
     <t>32220</t>
   </si>
   <si>
@@ -1360,10 +1360,10 @@
     <t>Construction policy and administrative management</t>
   </si>
   <si>
+    <t>Construction</t>
+  </si>
+  <si>
     <t>323</t>
-  </si>
-  <si>
-    <t>Construction</t>
   </si>
   <si>
     <t>33110</t>
@@ -2166,10 +2166,10 @@
         <v>9</v>
       </c>
       <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
         <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
       </c>
       <c r="F6" t="s">
         <v>23</v>
@@ -2189,10 +2189,10 @@
         <v>9</v>
       </c>
       <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
         <v>22</v>
-      </c>
-      <c r="E7" t="s">
-        <v>11</v>
       </c>
       <c r="F7" t="s">
         <v>23</v>
@@ -2212,10 +2212,10 @@
         <v>9</v>
       </c>
       <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
         <v>22</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
       </c>
       <c r="F8" t="s">
         <v>23</v>
@@ -2235,10 +2235,10 @@
         <v>9</v>
       </c>
       <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
         <v>22</v>
-      </c>
-      <c r="E9" t="s">
-        <v>11</v>
       </c>
       <c r="F9" t="s">
         <v>23</v>
@@ -2258,10 +2258,10 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
         <v>32</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
       </c>
       <c r="F10" t="s">
         <v>33</v>
@@ -2281,10 +2281,10 @@
         <v>9</v>
       </c>
       <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
         <v>32</v>
-      </c>
-      <c r="E11" t="s">
-        <v>11</v>
       </c>
       <c r="F11" t="s">
         <v>33</v>
@@ -2304,10 +2304,10 @@
         <v>9</v>
       </c>
       <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
         <v>38</v>
-      </c>
-      <c r="E12" t="s">
-        <v>11</v>
       </c>
       <c r="F12" t="s">
         <v>39</v>
@@ -2327,10 +2327,10 @@
         <v>9</v>
       </c>
       <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
         <v>38</v>
-      </c>
-      <c r="E13" t="s">
-        <v>11</v>
       </c>
       <c r="F13" t="s">
         <v>39</v>
@@ -2442,10 +2442,10 @@
         <v>9</v>
       </c>
       <c r="D18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" t="s">
         <v>56</v>
-      </c>
-      <c r="E18" t="s">
-        <v>45</v>
       </c>
       <c r="F18" t="s">
         <v>57</v>
@@ -2465,10 +2465,10 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" t="s">
         <v>56</v>
-      </c>
-      <c r="E19" t="s">
-        <v>45</v>
       </c>
       <c r="F19" t="s">
         <v>57</v>
@@ -2488,10 +2488,10 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" t="s">
         <v>56</v>
-      </c>
-      <c r="E20" t="s">
-        <v>45</v>
       </c>
       <c r="F20" t="s">
         <v>57</v>
@@ -2511,10 +2511,10 @@
         <v>9</v>
       </c>
       <c r="D21" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" t="s">
         <v>56</v>
-      </c>
-      <c r="E21" t="s">
-        <v>45</v>
       </c>
       <c r="F21" t="s">
         <v>57</v>
@@ -2534,10 +2534,10 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" t="s">
         <v>56</v>
-      </c>
-      <c r="E22" t="s">
-        <v>45</v>
       </c>
       <c r="F22" t="s">
         <v>57</v>
@@ -2557,10 +2557,10 @@
         <v>9</v>
       </c>
       <c r="D23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" t="s">
         <v>56</v>
-      </c>
-      <c r="E23" t="s">
-        <v>45</v>
       </c>
       <c r="F23" t="s">
         <v>57</v>
@@ -2580,10 +2580,10 @@
         <v>9</v>
       </c>
       <c r="D24" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" t="s">
         <v>56</v>
-      </c>
-      <c r="E24" t="s">
-        <v>45</v>
       </c>
       <c r="F24" t="s">
         <v>57</v>
@@ -2603,10 +2603,10 @@
         <v>9</v>
       </c>
       <c r="D25" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" t="s">
         <v>56</v>
-      </c>
-      <c r="E25" t="s">
-        <v>45</v>
       </c>
       <c r="F25" t="s">
         <v>57</v>
@@ -2626,10 +2626,10 @@
         <v>9</v>
       </c>
       <c r="D26" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" t="s">
         <v>74</v>
-      </c>
-      <c r="E26" t="s">
-        <v>45</v>
       </c>
       <c r="F26" t="s">
         <v>75</v>
@@ -2649,10 +2649,10 @@
         <v>9</v>
       </c>
       <c r="D27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" t="s">
         <v>74</v>
-      </c>
-      <c r="E27" t="s">
-        <v>45</v>
       </c>
       <c r="F27" t="s">
         <v>75</v>
@@ -2672,10 +2672,10 @@
         <v>9</v>
       </c>
       <c r="D28" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" t="s">
         <v>74</v>
-      </c>
-      <c r="E28" t="s">
-        <v>45</v>
       </c>
       <c r="F28" t="s">
         <v>75</v>
@@ -2695,10 +2695,10 @@
         <v>9</v>
       </c>
       <c r="D29" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" t="s">
         <v>74</v>
-      </c>
-      <c r="E29" t="s">
-        <v>45</v>
       </c>
       <c r="F29" t="s">
         <v>75</v>
@@ -2718,10 +2718,10 @@
         <v>9</v>
       </c>
       <c r="D30" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" t="s">
         <v>74</v>
-      </c>
-      <c r="E30" t="s">
-        <v>45</v>
       </c>
       <c r="F30" t="s">
         <v>75</v>
@@ -2741,10 +2741,10 @@
         <v>9</v>
       </c>
       <c r="D31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" t="s">
         <v>74</v>
-      </c>
-      <c r="E31" t="s">
-        <v>45</v>
       </c>
       <c r="F31" t="s">
         <v>75</v>
@@ -2770,10 +2770,10 @@
         <v>89</v>
       </c>
       <c r="F32" t="s">
+        <v>88</v>
+      </c>
+      <c r="G32" t="s">
         <v>89</v>
-      </c>
-      <c r="G32" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2793,10 +2793,10 @@
         <v>89</v>
       </c>
       <c r="F33" t="s">
+        <v>88</v>
+      </c>
+      <c r="G33" t="s">
         <v>89</v>
-      </c>
-      <c r="G33" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2816,10 +2816,10 @@
         <v>89</v>
       </c>
       <c r="F34" t="s">
+        <v>88</v>
+      </c>
+      <c r="G34" t="s">
         <v>89</v>
-      </c>
-      <c r="G34" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -2839,10 +2839,10 @@
         <v>89</v>
       </c>
       <c r="F35" t="s">
+        <v>88</v>
+      </c>
+      <c r="G35" t="s">
         <v>89</v>
-      </c>
-      <c r="G35" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -2862,10 +2862,10 @@
         <v>89</v>
       </c>
       <c r="F36" t="s">
+        <v>88</v>
+      </c>
+      <c r="G36" t="s">
         <v>89</v>
-      </c>
-      <c r="G36" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2885,10 +2885,10 @@
         <v>101</v>
       </c>
       <c r="F37" t="s">
+        <v>100</v>
+      </c>
+      <c r="G37" t="s">
         <v>101</v>
-      </c>
-      <c r="G37" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -2908,10 +2908,10 @@
         <v>101</v>
       </c>
       <c r="F38" t="s">
+        <v>100</v>
+      </c>
+      <c r="G38" t="s">
         <v>101</v>
-      </c>
-      <c r="G38" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -2931,10 +2931,10 @@
         <v>101</v>
       </c>
       <c r="F39" t="s">
+        <v>100</v>
+      </c>
+      <c r="G39" t="s">
         <v>101</v>
-      </c>
-      <c r="G39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2954,10 +2954,10 @@
         <v>101</v>
       </c>
       <c r="F40" t="s">
+        <v>100</v>
+      </c>
+      <c r="G40" t="s">
         <v>101</v>
-      </c>
-      <c r="G40" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -2977,10 +2977,10 @@
         <v>101</v>
       </c>
       <c r="F41" t="s">
+        <v>100</v>
+      </c>
+      <c r="G41" t="s">
         <v>101</v>
-      </c>
-      <c r="G41" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -3000,10 +3000,10 @@
         <v>101</v>
       </c>
       <c r="F42" t="s">
+        <v>100</v>
+      </c>
+      <c r="G42" t="s">
         <v>101</v>
-      </c>
-      <c r="G42" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -3023,10 +3023,10 @@
         <v>101</v>
       </c>
       <c r="F43" t="s">
+        <v>100</v>
+      </c>
+      <c r="G43" t="s">
         <v>101</v>
-      </c>
-      <c r="G43" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -3046,10 +3046,10 @@
         <v>101</v>
       </c>
       <c r="F44" t="s">
+        <v>100</v>
+      </c>
+      <c r="G44" t="s">
         <v>101</v>
-      </c>
-      <c r="G44" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -3069,10 +3069,10 @@
         <v>101</v>
       </c>
       <c r="F45" t="s">
+        <v>100</v>
+      </c>
+      <c r="G45" t="s">
         <v>101</v>
-      </c>
-      <c r="G45" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -3092,10 +3092,10 @@
         <v>101</v>
       </c>
       <c r="F46" t="s">
+        <v>100</v>
+      </c>
+      <c r="G46" t="s">
         <v>101</v>
-      </c>
-      <c r="G46" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -3115,10 +3115,10 @@
         <v>101</v>
       </c>
       <c r="F47" t="s">
+        <v>100</v>
+      </c>
+      <c r="G47" t="s">
         <v>101</v>
-      </c>
-      <c r="G47" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -3500,10 +3500,10 @@
         <v>9</v>
       </c>
       <c r="D64" t="s">
+        <v>124</v>
+      </c>
+      <c r="E64" t="s">
         <v>160</v>
-      </c>
-      <c r="E64" t="s">
-        <v>125</v>
       </c>
       <c r="F64" t="s">
         <v>161</v>
@@ -3523,10 +3523,10 @@
         <v>9</v>
       </c>
       <c r="D65" t="s">
+        <v>124</v>
+      </c>
+      <c r="E65" t="s">
         <v>160</v>
-      </c>
-      <c r="E65" t="s">
-        <v>125</v>
       </c>
       <c r="F65" t="s">
         <v>161</v>
@@ -3546,10 +3546,10 @@
         <v>9</v>
       </c>
       <c r="D66" t="s">
+        <v>124</v>
+      </c>
+      <c r="E66" t="s">
         <v>160</v>
-      </c>
-      <c r="E66" t="s">
-        <v>125</v>
       </c>
       <c r="F66" t="s">
         <v>161</v>
@@ -3569,10 +3569,10 @@
         <v>9</v>
       </c>
       <c r="D67" t="s">
+        <v>124</v>
+      </c>
+      <c r="E67" t="s">
         <v>160</v>
-      </c>
-      <c r="E67" t="s">
-        <v>125</v>
       </c>
       <c r="F67" t="s">
         <v>161</v>
@@ -3592,10 +3592,10 @@
         <v>9</v>
       </c>
       <c r="D68" t="s">
+        <v>124</v>
+      </c>
+      <c r="E68" t="s">
         <v>160</v>
-      </c>
-      <c r="E68" t="s">
-        <v>125</v>
       </c>
       <c r="F68" t="s">
         <v>161</v>
@@ -3615,10 +3615,10 @@
         <v>9</v>
       </c>
       <c r="D69" t="s">
+        <v>124</v>
+      </c>
+      <c r="E69" t="s">
         <v>160</v>
-      </c>
-      <c r="E69" t="s">
-        <v>125</v>
       </c>
       <c r="F69" t="s">
         <v>161</v>
@@ -3644,10 +3644,10 @@
         <v>175</v>
       </c>
       <c r="F70" t="s">
+        <v>174</v>
+      </c>
+      <c r="G70" t="s">
         <v>175</v>
-      </c>
-      <c r="G70" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -3667,10 +3667,10 @@
         <v>175</v>
       </c>
       <c r="F71" t="s">
+        <v>174</v>
+      </c>
+      <c r="G71" t="s">
         <v>175</v>
-      </c>
-      <c r="G71" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3690,10 +3690,10 @@
         <v>175</v>
       </c>
       <c r="F72" t="s">
+        <v>174</v>
+      </c>
+      <c r="G72" t="s">
         <v>175</v>
-      </c>
-      <c r="G72" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3713,10 +3713,10 @@
         <v>175</v>
       </c>
       <c r="F73" t="s">
+        <v>174</v>
+      </c>
+      <c r="G73" t="s">
         <v>175</v>
-      </c>
-      <c r="G73" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -3736,10 +3736,10 @@
         <v>175</v>
       </c>
       <c r="F74" t="s">
+        <v>174</v>
+      </c>
+      <c r="G74" t="s">
         <v>175</v>
-      </c>
-      <c r="G74" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -3759,10 +3759,10 @@
         <v>175</v>
       </c>
       <c r="F75" t="s">
+        <v>174</v>
+      </c>
+      <c r="G75" t="s">
         <v>175</v>
-      </c>
-      <c r="G75" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -3782,10 +3782,10 @@
         <v>175</v>
       </c>
       <c r="F76" t="s">
+        <v>174</v>
+      </c>
+      <c r="G76" t="s">
         <v>175</v>
-      </c>
-      <c r="G76" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -3805,10 +3805,10 @@
         <v>175</v>
       </c>
       <c r="F77" t="s">
+        <v>174</v>
+      </c>
+      <c r="G77" t="s">
         <v>175</v>
-      </c>
-      <c r="G77" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -3828,10 +3828,10 @@
         <v>175</v>
       </c>
       <c r="F78" t="s">
+        <v>174</v>
+      </c>
+      <c r="G78" t="s">
         <v>175</v>
-      </c>
-      <c r="G78" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -3851,10 +3851,10 @@
         <v>175</v>
       </c>
       <c r="F79" t="s">
+        <v>174</v>
+      </c>
+      <c r="G79" t="s">
         <v>175</v>
-      </c>
-      <c r="G79" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -3874,10 +3874,10 @@
         <v>175</v>
       </c>
       <c r="F80" t="s">
+        <v>174</v>
+      </c>
+      <c r="G80" t="s">
         <v>175</v>
-      </c>
-      <c r="G80" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -3897,10 +3897,10 @@
         <v>199</v>
       </c>
       <c r="F81" t="s">
+        <v>198</v>
+      </c>
+      <c r="G81" t="s">
         <v>199</v>
-      </c>
-      <c r="G81" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -3920,10 +3920,10 @@
         <v>199</v>
       </c>
       <c r="F82" t="s">
+        <v>198</v>
+      </c>
+      <c r="G82" t="s">
         <v>199</v>
-      </c>
-      <c r="G82" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -3943,10 +3943,10 @@
         <v>199</v>
       </c>
       <c r="F83" t="s">
+        <v>198</v>
+      </c>
+      <c r="G83" t="s">
         <v>199</v>
-      </c>
-      <c r="G83" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -3966,10 +3966,10 @@
         <v>199</v>
       </c>
       <c r="F84" t="s">
+        <v>198</v>
+      </c>
+      <c r="G84" t="s">
         <v>199</v>
-      </c>
-      <c r="G84" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -3989,10 +3989,10 @@
         <v>199</v>
       </c>
       <c r="F85" t="s">
+        <v>198</v>
+      </c>
+      <c r="G85" t="s">
         <v>199</v>
-      </c>
-      <c r="G85" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -4012,10 +4012,10 @@
         <v>199</v>
       </c>
       <c r="F86" t="s">
+        <v>198</v>
+      </c>
+      <c r="G86" t="s">
         <v>199</v>
-      </c>
-      <c r="G86" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -4035,10 +4035,10 @@
         <v>199</v>
       </c>
       <c r="F87" t="s">
+        <v>198</v>
+      </c>
+      <c r="G87" t="s">
         <v>199</v>
-      </c>
-      <c r="G87" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -4058,10 +4058,10 @@
         <v>215</v>
       </c>
       <c r="F88" t="s">
+        <v>214</v>
+      </c>
+      <c r="G88" t="s">
         <v>215</v>
-      </c>
-      <c r="G88" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -4081,10 +4081,10 @@
         <v>215</v>
       </c>
       <c r="F89" t="s">
+        <v>214</v>
+      </c>
+      <c r="G89" t="s">
         <v>215</v>
-      </c>
-      <c r="G89" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -4104,10 +4104,10 @@
         <v>215</v>
       </c>
       <c r="F90" t="s">
+        <v>214</v>
+      </c>
+      <c r="G90" t="s">
         <v>215</v>
-      </c>
-      <c r="G90" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -4127,10 +4127,10 @@
         <v>215</v>
       </c>
       <c r="F91" t="s">
+        <v>214</v>
+      </c>
+      <c r="G91" t="s">
         <v>215</v>
-      </c>
-      <c r="G91" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -4236,10 +4236,10 @@
         <v>9</v>
       </c>
       <c r="D96" t="s">
+        <v>224</v>
+      </c>
+      <c r="E96" t="s">
         <v>236</v>
-      </c>
-      <c r="E96" t="s">
-        <v>225</v>
       </c>
       <c r="F96" t="s">
         <v>237</v>
@@ -4259,10 +4259,10 @@
         <v>9</v>
       </c>
       <c r="D97" t="s">
+        <v>224</v>
+      </c>
+      <c r="E97" t="s">
         <v>236</v>
-      </c>
-      <c r="E97" t="s">
-        <v>225</v>
       </c>
       <c r="F97" t="s">
         <v>237</v>
@@ -4282,10 +4282,10 @@
         <v>9</v>
       </c>
       <c r="D98" t="s">
+        <v>224</v>
+      </c>
+      <c r="E98" t="s">
         <v>236</v>
-      </c>
-      <c r="E98" t="s">
-        <v>225</v>
       </c>
       <c r="F98" t="s">
         <v>237</v>
@@ -4305,10 +4305,10 @@
         <v>9</v>
       </c>
       <c r="D99" t="s">
+        <v>224</v>
+      </c>
+      <c r="E99" t="s">
         <v>236</v>
-      </c>
-      <c r="E99" t="s">
-        <v>225</v>
       </c>
       <c r="F99" t="s">
         <v>237</v>
@@ -4328,10 +4328,10 @@
         <v>9</v>
       </c>
       <c r="D100" t="s">
+        <v>224</v>
+      </c>
+      <c r="E100" t="s">
         <v>236</v>
-      </c>
-      <c r="E100" t="s">
-        <v>225</v>
       </c>
       <c r="F100" t="s">
         <v>237</v>
@@ -4351,10 +4351,10 @@
         <v>9</v>
       </c>
       <c r="D101" t="s">
+        <v>224</v>
+      </c>
+      <c r="E101" t="s">
         <v>236</v>
-      </c>
-      <c r="E101" t="s">
-        <v>225</v>
       </c>
       <c r="F101" t="s">
         <v>237</v>
@@ -4374,10 +4374,10 @@
         <v>9</v>
       </c>
       <c r="D102" t="s">
+        <v>224</v>
+      </c>
+      <c r="E102" t="s">
         <v>236</v>
-      </c>
-      <c r="E102" t="s">
-        <v>225</v>
       </c>
       <c r="F102" t="s">
         <v>237</v>
@@ -4397,10 +4397,10 @@
         <v>9</v>
       </c>
       <c r="D103" t="s">
+        <v>224</v>
+      </c>
+      <c r="E103" t="s">
         <v>236</v>
-      </c>
-      <c r="E103" t="s">
-        <v>225</v>
       </c>
       <c r="F103" t="s">
         <v>237</v>
@@ -4420,10 +4420,10 @@
         <v>9</v>
       </c>
       <c r="D104" t="s">
+        <v>224</v>
+      </c>
+      <c r="E104" t="s">
         <v>236</v>
-      </c>
-      <c r="E104" t="s">
-        <v>225</v>
       </c>
       <c r="F104" t="s">
         <v>237</v>
@@ -4443,10 +4443,10 @@
         <v>9</v>
       </c>
       <c r="D105" t="s">
+        <v>224</v>
+      </c>
+      <c r="E105" t="s">
         <v>256</v>
-      </c>
-      <c r="E105" t="s">
-        <v>225</v>
       </c>
       <c r="F105" t="s">
         <v>257</v>
@@ -4466,10 +4466,10 @@
         <v>9</v>
       </c>
       <c r="D106" t="s">
+        <v>224</v>
+      </c>
+      <c r="E106" t="s">
         <v>256</v>
-      </c>
-      <c r="E106" t="s">
-        <v>225</v>
       </c>
       <c r="F106" t="s">
         <v>257</v>
@@ -4489,10 +4489,10 @@
         <v>9</v>
       </c>
       <c r="D107" t="s">
+        <v>224</v>
+      </c>
+      <c r="E107" t="s">
         <v>256</v>
-      </c>
-      <c r="E107" t="s">
-        <v>225</v>
       </c>
       <c r="F107" t="s">
         <v>257</v>
@@ -4512,10 +4512,10 @@
         <v>9</v>
       </c>
       <c r="D108" t="s">
+        <v>224</v>
+      </c>
+      <c r="E108" t="s">
         <v>256</v>
-      </c>
-      <c r="E108" t="s">
-        <v>225</v>
       </c>
       <c r="F108" t="s">
         <v>257</v>
@@ -4535,10 +4535,10 @@
         <v>9</v>
       </c>
       <c r="D109" t="s">
+        <v>224</v>
+      </c>
+      <c r="E109" t="s">
         <v>256</v>
-      </c>
-      <c r="E109" t="s">
-        <v>225</v>
       </c>
       <c r="F109" t="s">
         <v>257</v>
@@ -4558,10 +4558,10 @@
         <v>9</v>
       </c>
       <c r="D110" t="s">
+        <v>224</v>
+      </c>
+      <c r="E110" t="s">
         <v>256</v>
-      </c>
-      <c r="E110" t="s">
-        <v>225</v>
       </c>
       <c r="F110" t="s">
         <v>257</v>
@@ -4581,10 +4581,10 @@
         <v>9</v>
       </c>
       <c r="D111" t="s">
+        <v>224</v>
+      </c>
+      <c r="E111" t="s">
         <v>270</v>
-      </c>
-      <c r="E111" t="s">
-        <v>225</v>
       </c>
       <c r="F111" t="s">
         <v>271</v>
@@ -4604,10 +4604,10 @@
         <v>9</v>
       </c>
       <c r="D112" t="s">
+        <v>224</v>
+      </c>
+      <c r="E112" t="s">
         <v>274</v>
-      </c>
-      <c r="E112" t="s">
-        <v>225</v>
       </c>
       <c r="F112" t="s">
         <v>275</v>
@@ -4627,10 +4627,10 @@
         <v>9</v>
       </c>
       <c r="D113" t="s">
+        <v>224</v>
+      </c>
+      <c r="E113" t="s">
         <v>278</v>
-      </c>
-      <c r="E113" t="s">
-        <v>225</v>
       </c>
       <c r="F113" t="s">
         <v>279</v>
@@ -4650,10 +4650,10 @@
         <v>9</v>
       </c>
       <c r="D114" t="s">
+        <v>224</v>
+      </c>
+      <c r="E114" t="s">
         <v>278</v>
-      </c>
-      <c r="E114" t="s">
-        <v>225</v>
       </c>
       <c r="F114" t="s">
         <v>279</v>
@@ -4673,10 +4673,10 @@
         <v>9</v>
       </c>
       <c r="D115" t="s">
+        <v>224</v>
+      </c>
+      <c r="E115" t="s">
         <v>278</v>
-      </c>
-      <c r="E115" t="s">
-        <v>225</v>
       </c>
       <c r="F115" t="s">
         <v>279</v>
@@ -4696,10 +4696,10 @@
         <v>9</v>
       </c>
       <c r="D116" t="s">
+        <v>224</v>
+      </c>
+      <c r="E116" t="s">
         <v>278</v>
-      </c>
-      <c r="E116" t="s">
-        <v>225</v>
       </c>
       <c r="F116" t="s">
         <v>279</v>
@@ -4719,10 +4719,10 @@
         <v>9</v>
       </c>
       <c r="D117" t="s">
+        <v>224</v>
+      </c>
+      <c r="E117" t="s">
         <v>278</v>
-      </c>
-      <c r="E117" t="s">
-        <v>225</v>
       </c>
       <c r="F117" t="s">
         <v>279</v>
@@ -4742,10 +4742,10 @@
         <v>9</v>
       </c>
       <c r="D118" t="s">
+        <v>224</v>
+      </c>
+      <c r="E118" t="s">
         <v>278</v>
-      </c>
-      <c r="E118" t="s">
-        <v>225</v>
       </c>
       <c r="F118" t="s">
         <v>279</v>
@@ -4765,10 +4765,10 @@
         <v>9</v>
       </c>
       <c r="D119" t="s">
+        <v>224</v>
+      </c>
+      <c r="E119" t="s">
         <v>278</v>
-      </c>
-      <c r="E119" t="s">
-        <v>225</v>
       </c>
       <c r="F119" t="s">
         <v>279</v>
@@ -4794,10 +4794,10 @@
         <v>295</v>
       </c>
       <c r="F120" t="s">
+        <v>294</v>
+      </c>
+      <c r="G120" t="s">
         <v>295</v>
-      </c>
-      <c r="G120" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -4817,10 +4817,10 @@
         <v>295</v>
       </c>
       <c r="F121" t="s">
+        <v>294</v>
+      </c>
+      <c r="G121" t="s">
         <v>295</v>
-      </c>
-      <c r="G121" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -4840,10 +4840,10 @@
         <v>295</v>
       </c>
       <c r="F122" t="s">
+        <v>294</v>
+      </c>
+      <c r="G122" t="s">
         <v>295</v>
-      </c>
-      <c r="G122" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -4863,10 +4863,10 @@
         <v>295</v>
       </c>
       <c r="F123" t="s">
+        <v>294</v>
+      </c>
+      <c r="G123" t="s">
         <v>295</v>
-      </c>
-      <c r="G123" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -4886,10 +4886,10 @@
         <v>295</v>
       </c>
       <c r="F124" t="s">
+        <v>294</v>
+      </c>
+      <c r="G124" t="s">
         <v>295</v>
-      </c>
-      <c r="G124" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="125" spans="1:7">
@@ -4909,10 +4909,10 @@
         <v>295</v>
       </c>
       <c r="F125" t="s">
+        <v>294</v>
+      </c>
+      <c r="G125" t="s">
         <v>295</v>
-      </c>
-      <c r="G125" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -4932,10 +4932,10 @@
         <v>309</v>
       </c>
       <c r="F126" t="s">
+        <v>308</v>
+      </c>
+      <c r="G126" t="s">
         <v>309</v>
-      </c>
-      <c r="G126" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -4955,10 +4955,10 @@
         <v>309</v>
       </c>
       <c r="F127" t="s">
+        <v>308</v>
+      </c>
+      <c r="G127" t="s">
         <v>309</v>
-      </c>
-      <c r="G127" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -4978,10 +4978,10 @@
         <v>309</v>
       </c>
       <c r="F128" t="s">
+        <v>308</v>
+      </c>
+      <c r="G128" t="s">
         <v>309</v>
-      </c>
-      <c r="G128" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="129" spans="1:7">
@@ -5001,10 +5001,10 @@
         <v>309</v>
       </c>
       <c r="F129" t="s">
+        <v>308</v>
+      </c>
+      <c r="G129" t="s">
         <v>309</v>
-      </c>
-      <c r="G129" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="130" spans="1:7">
@@ -5432,10 +5432,10 @@
         <v>9</v>
       </c>
       <c r="D148" t="s">
+        <v>318</v>
+      </c>
+      <c r="E148" t="s">
         <v>358</v>
-      </c>
-      <c r="E148" t="s">
-        <v>319</v>
       </c>
       <c r="F148" t="s">
         <v>359</v>
@@ -5455,10 +5455,10 @@
         <v>9</v>
       </c>
       <c r="D149" t="s">
+        <v>318</v>
+      </c>
+      <c r="E149" t="s">
         <v>358</v>
-      </c>
-      <c r="E149" t="s">
-        <v>319</v>
       </c>
       <c r="F149" t="s">
         <v>359</v>
@@ -5478,10 +5478,10 @@
         <v>9</v>
       </c>
       <c r="D150" t="s">
+        <v>318</v>
+      </c>
+      <c r="E150" t="s">
         <v>358</v>
-      </c>
-      <c r="E150" t="s">
-        <v>319</v>
       </c>
       <c r="F150" t="s">
         <v>359</v>
@@ -5501,10 +5501,10 @@
         <v>9</v>
       </c>
       <c r="D151" t="s">
+        <v>318</v>
+      </c>
+      <c r="E151" t="s">
         <v>358</v>
-      </c>
-      <c r="E151" t="s">
-        <v>319</v>
       </c>
       <c r="F151" t="s">
         <v>359</v>
@@ -5524,10 +5524,10 @@
         <v>9</v>
       </c>
       <c r="D152" t="s">
+        <v>318</v>
+      </c>
+      <c r="E152" t="s">
         <v>358</v>
-      </c>
-      <c r="E152" t="s">
-        <v>319</v>
       </c>
       <c r="F152" t="s">
         <v>359</v>
@@ -5547,10 +5547,10 @@
         <v>9</v>
       </c>
       <c r="D153" t="s">
+        <v>318</v>
+      </c>
+      <c r="E153" t="s">
         <v>358</v>
-      </c>
-      <c r="E153" t="s">
-        <v>319</v>
       </c>
       <c r="F153" t="s">
         <v>359</v>
@@ -5570,10 +5570,10 @@
         <v>9</v>
       </c>
       <c r="D154" t="s">
+        <v>318</v>
+      </c>
+      <c r="E154" t="s">
         <v>372</v>
-      </c>
-      <c r="E154" t="s">
-        <v>319</v>
       </c>
       <c r="F154" t="s">
         <v>373</v>
@@ -5593,10 +5593,10 @@
         <v>9</v>
       </c>
       <c r="D155" t="s">
+        <v>318</v>
+      </c>
+      <c r="E155" t="s">
         <v>372</v>
-      </c>
-      <c r="E155" t="s">
-        <v>319</v>
       </c>
       <c r="F155" t="s">
         <v>373</v>
@@ -5616,10 +5616,10 @@
         <v>9</v>
       </c>
       <c r="D156" t="s">
+        <v>318</v>
+      </c>
+      <c r="E156" t="s">
         <v>372</v>
-      </c>
-      <c r="E156" t="s">
-        <v>319</v>
       </c>
       <c r="F156" t="s">
         <v>373</v>
@@ -5639,10 +5639,10 @@
         <v>9</v>
       </c>
       <c r="D157" t="s">
+        <v>318</v>
+      </c>
+      <c r="E157" t="s">
         <v>372</v>
-      </c>
-      <c r="E157" t="s">
-        <v>319</v>
       </c>
       <c r="F157" t="s">
         <v>373</v>
@@ -5662,10 +5662,10 @@
         <v>9</v>
       </c>
       <c r="D158" t="s">
+        <v>318</v>
+      </c>
+      <c r="E158" t="s">
         <v>372</v>
-      </c>
-      <c r="E158" t="s">
-        <v>319</v>
       </c>
       <c r="F158" t="s">
         <v>373</v>
@@ -6122,10 +6122,10 @@
         <v>9</v>
       </c>
       <c r="D178" t="s">
+        <v>384</v>
+      </c>
+      <c r="E178" t="s">
         <v>426</v>
-      </c>
-      <c r="E178" t="s">
-        <v>385</v>
       </c>
       <c r="F178" t="s">
         <v>427</v>
@@ -6145,10 +6145,10 @@
         <v>9</v>
       </c>
       <c r="D179" t="s">
+        <v>384</v>
+      </c>
+      <c r="E179" t="s">
         <v>426</v>
-      </c>
-      <c r="E179" t="s">
-        <v>385</v>
       </c>
       <c r="F179" t="s">
         <v>427</v>
@@ -6168,10 +6168,10 @@
         <v>9</v>
       </c>
       <c r="D180" t="s">
+        <v>384</v>
+      </c>
+      <c r="E180" t="s">
         <v>426</v>
-      </c>
-      <c r="E180" t="s">
-        <v>385</v>
       </c>
       <c r="F180" t="s">
         <v>427</v>
@@ -6191,10 +6191,10 @@
         <v>9</v>
       </c>
       <c r="D181" t="s">
+        <v>384</v>
+      </c>
+      <c r="E181" t="s">
         <v>426</v>
-      </c>
-      <c r="E181" t="s">
-        <v>385</v>
       </c>
       <c r="F181" t="s">
         <v>427</v>
@@ -6214,10 +6214,10 @@
         <v>9</v>
       </c>
       <c r="D182" t="s">
+        <v>384</v>
+      </c>
+      <c r="E182" t="s">
         <v>426</v>
-      </c>
-      <c r="E182" t="s">
-        <v>385</v>
       </c>
       <c r="F182" t="s">
         <v>427</v>
@@ -6237,10 +6237,10 @@
         <v>9</v>
       </c>
       <c r="D183" t="s">
+        <v>384</v>
+      </c>
+      <c r="E183" t="s">
         <v>426</v>
-      </c>
-      <c r="E183" t="s">
-        <v>385</v>
       </c>
       <c r="F183" t="s">
         <v>427</v>
@@ -6260,10 +6260,10 @@
         <v>9</v>
       </c>
       <c r="D184" t="s">
+        <v>384</v>
+      </c>
+      <c r="E184" t="s">
         <v>426</v>
-      </c>
-      <c r="E184" t="s">
-        <v>385</v>
       </c>
       <c r="F184" t="s">
         <v>427</v>
@@ -6283,10 +6283,10 @@
         <v>9</v>
       </c>
       <c r="D185" t="s">
+        <v>384</v>
+      </c>
+      <c r="E185" t="s">
         <v>426</v>
-      </c>
-      <c r="E185" t="s">
-        <v>385</v>
       </c>
       <c r="F185" t="s">
         <v>427</v>
@@ -6306,10 +6306,10 @@
         <v>9</v>
       </c>
       <c r="D186" t="s">
+        <v>384</v>
+      </c>
+      <c r="E186" t="s">
         <v>426</v>
-      </c>
-      <c r="E186" t="s">
-        <v>385</v>
       </c>
       <c r="F186" t="s">
         <v>427</v>
@@ -6329,10 +6329,10 @@
         <v>9</v>
       </c>
       <c r="D187" t="s">
+        <v>384</v>
+      </c>
+      <c r="E187" t="s">
         <v>426</v>
-      </c>
-      <c r="E187" t="s">
-        <v>385</v>
       </c>
       <c r="F187" t="s">
         <v>427</v>
@@ -6352,10 +6352,10 @@
         <v>9</v>
       </c>
       <c r="D188" t="s">
+        <v>384</v>
+      </c>
+      <c r="E188" t="s">
         <v>448</v>
-      </c>
-      <c r="E188" t="s">
-        <v>385</v>
       </c>
       <c r="F188" t="s">
         <v>449</v>
@@ -6381,10 +6381,10 @@
         <v>453</v>
       </c>
       <c r="F189" t="s">
+        <v>452</v>
+      </c>
+      <c r="G189" t="s">
         <v>453</v>
-      </c>
-      <c r="G189" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="190" spans="1:7">
@@ -6404,10 +6404,10 @@
         <v>453</v>
       </c>
       <c r="F190" t="s">
+        <v>452</v>
+      </c>
+      <c r="G190" t="s">
         <v>453</v>
-      </c>
-      <c r="G190" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="191" spans="1:7">
@@ -6427,10 +6427,10 @@
         <v>453</v>
       </c>
       <c r="F191" t="s">
+        <v>452</v>
+      </c>
+      <c r="G191" t="s">
         <v>453</v>
-      </c>
-      <c r="G191" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="192" spans="1:7">
@@ -6450,10 +6450,10 @@
         <v>453</v>
       </c>
       <c r="F192" t="s">
+        <v>452</v>
+      </c>
+      <c r="G192" t="s">
         <v>453</v>
-      </c>
-      <c r="G192" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="193" spans="1:7">
@@ -6473,10 +6473,10 @@
         <v>453</v>
       </c>
       <c r="F193" t="s">
+        <v>452</v>
+      </c>
+      <c r="G193" t="s">
         <v>453</v>
-      </c>
-      <c r="G193" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="194" spans="1:7">
@@ -6496,10 +6496,10 @@
         <v>453</v>
       </c>
       <c r="F194" t="s">
+        <v>452</v>
+      </c>
+      <c r="G194" t="s">
         <v>453</v>
-      </c>
-      <c r="G194" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="195" spans="1:7">
@@ -6519,10 +6519,10 @@
         <v>467</v>
       </c>
       <c r="F195" t="s">
+        <v>466</v>
+      </c>
+      <c r="G195" t="s">
         <v>467</v>
-      </c>
-      <c r="G195" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="196" spans="1:7">
@@ -6542,10 +6542,10 @@
         <v>471</v>
       </c>
       <c r="F196" t="s">
+        <v>470</v>
+      </c>
+      <c r="G196" t="s">
         <v>471</v>
-      </c>
-      <c r="G196" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="197" spans="1:7">
@@ -6565,10 +6565,10 @@
         <v>471</v>
       </c>
       <c r="F197" t="s">
+        <v>470</v>
+      </c>
+      <c r="G197" t="s">
         <v>471</v>
-      </c>
-      <c r="G197" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="198" spans="1:7">
@@ -6588,10 +6588,10 @@
         <v>471</v>
       </c>
       <c r="F198" t="s">
+        <v>470</v>
+      </c>
+      <c r="G198" t="s">
         <v>471</v>
-      </c>
-      <c r="G198" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="199" spans="1:7">
@@ -6611,10 +6611,10 @@
         <v>471</v>
       </c>
       <c r="F199" t="s">
+        <v>470</v>
+      </c>
+      <c r="G199" t="s">
         <v>471</v>
-      </c>
-      <c r="G199" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="200" spans="1:7">
@@ -6634,10 +6634,10 @@
         <v>471</v>
       </c>
       <c r="F200" t="s">
+        <v>470</v>
+      </c>
+      <c r="G200" t="s">
         <v>471</v>
-      </c>
-      <c r="G200" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="201" spans="1:7">
@@ -6657,10 +6657,10 @@
         <v>471</v>
       </c>
       <c r="F201" t="s">
+        <v>470</v>
+      </c>
+      <c r="G201" t="s">
         <v>471</v>
-      </c>
-      <c r="G201" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="202" spans="1:7">
@@ -6680,10 +6680,10 @@
         <v>485</v>
       </c>
       <c r="F202" t="s">
+        <v>484</v>
+      </c>
+      <c r="G202" t="s">
         <v>485</v>
-      </c>
-      <c r="G202" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="203" spans="1:7">
@@ -6703,10 +6703,10 @@
         <v>485</v>
       </c>
       <c r="F203" t="s">
+        <v>484</v>
+      </c>
+      <c r="G203" t="s">
         <v>485</v>
-      </c>
-      <c r="G203" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="204" spans="1:7">
@@ -6726,10 +6726,10 @@
         <v>485</v>
       </c>
       <c r="F204" t="s">
+        <v>484</v>
+      </c>
+      <c r="G204" t="s">
         <v>485</v>
-      </c>
-      <c r="G204" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="205" spans="1:7">
@@ -6749,10 +6749,10 @@
         <v>485</v>
       </c>
       <c r="F205" t="s">
+        <v>484</v>
+      </c>
+      <c r="G205" t="s">
         <v>485</v>
-      </c>
-      <c r="G205" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="206" spans="1:7">
@@ -6772,10 +6772,10 @@
         <v>485</v>
       </c>
       <c r="F206" t="s">
+        <v>484</v>
+      </c>
+      <c r="G206" t="s">
         <v>485</v>
-      </c>
-      <c r="G206" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="207" spans="1:7">
@@ -6795,10 +6795,10 @@
         <v>485</v>
       </c>
       <c r="F207" t="s">
+        <v>484</v>
+      </c>
+      <c r="G207" t="s">
         <v>485</v>
-      </c>
-      <c r="G207" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="208" spans="1:7">
@@ -6818,10 +6818,10 @@
         <v>485</v>
       </c>
       <c r="F208" t="s">
+        <v>484</v>
+      </c>
+      <c r="G208" t="s">
         <v>485</v>
-      </c>
-      <c r="G208" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="209" spans="1:7">
@@ -6841,10 +6841,10 @@
         <v>485</v>
       </c>
       <c r="F209" t="s">
+        <v>484</v>
+      </c>
+      <c r="G209" t="s">
         <v>485</v>
-      </c>
-      <c r="G209" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="210" spans="1:7">
@@ -6864,10 +6864,10 @@
         <v>485</v>
       </c>
       <c r="F210" t="s">
+        <v>484</v>
+      </c>
+      <c r="G210" t="s">
         <v>485</v>
-      </c>
-      <c r="G210" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="211" spans="1:7">
@@ -6887,10 +6887,10 @@
         <v>485</v>
       </c>
       <c r="F211" t="s">
+        <v>484</v>
+      </c>
+      <c r="G211" t="s">
         <v>485</v>
-      </c>
-      <c r="G211" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="212" spans="1:7">
@@ -6910,10 +6910,10 @@
         <v>507</v>
       </c>
       <c r="F212" t="s">
+        <v>506</v>
+      </c>
+      <c r="G212" t="s">
         <v>507</v>
-      </c>
-      <c r="G212" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="213" spans="1:7">
@@ -6933,10 +6933,10 @@
         <v>511</v>
       </c>
       <c r="F213" t="s">
+        <v>510</v>
+      </c>
+      <c r="G213" t="s">
         <v>511</v>
-      </c>
-      <c r="G213" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="214" spans="1:7">
@@ -6956,10 +6956,10 @@
         <v>515</v>
       </c>
       <c r="F214" t="s">
+        <v>514</v>
+      </c>
+      <c r="G214" t="s">
         <v>515</v>
-      </c>
-      <c r="G214" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="215" spans="1:7">
@@ -6979,10 +6979,10 @@
         <v>515</v>
       </c>
       <c r="F215" t="s">
+        <v>514</v>
+      </c>
+      <c r="G215" t="s">
         <v>515</v>
-      </c>
-      <c r="G215" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="216" spans="1:7">
@@ -7002,10 +7002,10 @@
         <v>521</v>
       </c>
       <c r="F216" t="s">
+        <v>520</v>
+      </c>
+      <c r="G216" t="s">
         <v>521</v>
-      </c>
-      <c r="G216" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="217" spans="1:7">
@@ -7025,10 +7025,10 @@
         <v>521</v>
       </c>
       <c r="F217" t="s">
+        <v>520</v>
+      </c>
+      <c r="G217" t="s">
         <v>521</v>
-      </c>
-      <c r="G217" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="218" spans="1:7">
@@ -7048,10 +7048,10 @@
         <v>521</v>
       </c>
       <c r="F218" t="s">
+        <v>520</v>
+      </c>
+      <c r="G218" t="s">
         <v>521</v>
-      </c>
-      <c r="G218" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="219" spans="1:7">
@@ -7071,10 +7071,10 @@
         <v>521</v>
       </c>
       <c r="F219" t="s">
+        <v>520</v>
+      </c>
+      <c r="G219" t="s">
         <v>521</v>
-      </c>
-      <c r="G219" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -7094,10 +7094,10 @@
         <v>521</v>
       </c>
       <c r="F220" t="s">
+        <v>520</v>
+      </c>
+      <c r="G220" t="s">
         <v>521</v>
-      </c>
-      <c r="G220" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="221" spans="1:7">
@@ -7117,10 +7117,10 @@
         <v>521</v>
       </c>
       <c r="F221" t="s">
+        <v>520</v>
+      </c>
+      <c r="G221" t="s">
         <v>521</v>
-      </c>
-      <c r="G221" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="222" spans="1:7">
@@ -7140,10 +7140,10 @@
         <v>521</v>
       </c>
       <c r="F222" t="s">
+        <v>520</v>
+      </c>
+      <c r="G222" t="s">
         <v>521</v>
-      </c>
-      <c r="G222" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="223" spans="1:7">
@@ -7163,10 +7163,10 @@
         <v>537</v>
       </c>
       <c r="F223" t="s">
+        <v>536</v>
+      </c>
+      <c r="G223" t="s">
         <v>537</v>
-      </c>
-      <c r="G223" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="224" spans="1:7">
@@ -7186,10 +7186,10 @@
         <v>537</v>
       </c>
       <c r="F224" t="s">
+        <v>536</v>
+      </c>
+      <c r="G224" t="s">
         <v>537</v>
-      </c>
-      <c r="G224" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="225" spans="1:7">
@@ -7209,10 +7209,10 @@
         <v>537</v>
       </c>
       <c r="F225" t="s">
+        <v>536</v>
+      </c>
+      <c r="G225" t="s">
         <v>537</v>
-      </c>
-      <c r="G225" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="226" spans="1:7">
@@ -7232,10 +7232,10 @@
         <v>545</v>
       </c>
       <c r="F226" t="s">
+        <v>544</v>
+      </c>
+      <c r="G226" t="s">
         <v>545</v>
-      </c>
-      <c r="G226" t="s">
-        <v>544</v>
       </c>
     </row>
     <row r="227" spans="1:7">
@@ -7255,10 +7255,10 @@
         <v>549</v>
       </c>
       <c r="F227" t="s">
+        <v>548</v>
+      </c>
+      <c r="G227" t="s">
         <v>549</v>
-      </c>
-      <c r="G227" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="228" spans="1:7">
@@ -7278,10 +7278,10 @@
         <v>553</v>
       </c>
       <c r="F228" t="s">
+        <v>552</v>
+      </c>
+      <c r="G228" t="s">
         <v>553</v>
-      </c>
-      <c r="G228" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="229" spans="1:7">
@@ -7301,10 +7301,10 @@
         <v>557</v>
       </c>
       <c r="F229" t="s">
+        <v>556</v>
+      </c>
+      <c r="G229" t="s">
         <v>557</v>
-      </c>
-      <c r="G229" t="s">
-        <v>556</v>
       </c>
     </row>
     <row r="230" spans="1:7">
@@ -7324,10 +7324,10 @@
         <v>561</v>
       </c>
       <c r="F230" t="s">
+        <v>560</v>
+      </c>
+      <c r="G230" t="s">
         <v>561</v>
-      </c>
-      <c r="G230" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="231" spans="1:7">
@@ -7347,10 +7347,10 @@
         <v>561</v>
       </c>
       <c r="F231" t="s">
+        <v>560</v>
+      </c>
+      <c r="G231" t="s">
         <v>561</v>
-      </c>
-      <c r="G231" t="s">
-        <v>560</v>
       </c>
     </row>
   </sheetData>

</xml_diff>